<commit_message>
generate figure for inter model comparison
</commit_message>
<xml_diff>
--- a/inter_model_compare/Inter_model_Stat_results.xlsx
+++ b/inter_model_compare/Inter_model_Stat_results.xlsx
@@ -1236,16 +1236,16 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>16.5</v>
+        <v>52.5</v>
       </c>
       <c r="E28" t="n">
-        <v>0.007724233637416746</v>
+        <v>0.433197021484375</v>
       </c>
       <c r="F28" t="n">
-        <v>-3.010098070412778</v>
+        <v>-1.470387340513864</v>
       </c>
       <c r="G28" t="n">
-        <v>0.008790093097708975</v>
+        <v>0.1621208233067553</v>
       </c>
     </row>
     <row r="29">
@@ -1294,16 +1294,16 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>24.5</v>
+        <v>27</v>
       </c>
       <c r="E30" t="n">
-        <v>0.021392822265625</v>
+        <v>0.033538818359375</v>
       </c>
       <c r="F30" t="n">
-        <v>-1.664837300219328</v>
+        <v>2.129538870678781</v>
       </c>
       <c r="G30" t="n">
-        <v>0.1166883803046404</v>
+        <v>0.05018088582646035</v>
       </c>
     </row>
     <row r="31">
@@ -1323,16 +1323,16 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E31" t="n">
-        <v>1</v>
+        <v>0.010986328125</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>2.97869377386183</v>
       </c>
       <c r="G31" t="n">
-        <v>1</v>
+        <v>0.009370417962060751</v>
       </c>
     </row>
     <row r="32">
@@ -1410,16 +1410,16 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>33.5</v>
+        <v>7.5</v>
       </c>
       <c r="E34" t="n">
-        <v>0.07443137895800514</v>
+        <v>0.001754599535343804</v>
       </c>
       <c r="F34" t="n">
-        <v>-1.461552038022779</v>
+        <v>-3.110492647370015</v>
       </c>
       <c r="G34" t="n">
-        <v>0.164496220837515</v>
+        <v>0.007162047525193289</v>
       </c>
     </row>
     <row r="35">
@@ -1468,16 +1468,16 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>9.5</v>
+        <v>63.5</v>
       </c>
       <c r="E36" t="n">
-        <v>0.002478331942743607</v>
+        <v>0.815942129589875</v>
       </c>
       <c r="F36" t="n">
-        <v>2.7908305332692</v>
+        <v>-0.286192865876731</v>
       </c>
       <c r="G36" t="n">
-        <v>0.01371098595327495</v>
+        <v>0.7786451558117076</v>
       </c>
     </row>
     <row r="37">
@@ -1497,16 +1497,16 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E37" t="n">
-        <v>1</v>
+        <v>0.0004824029369617037</v>
       </c>
       <c r="F37" t="n">
-        <v>0</v>
+        <v>-3.902076292289889</v>
       </c>
       <c r="G37" t="n">
-        <v>1</v>
+        <v>0.001415222751478339</v>
       </c>
     </row>
     <row r="38">
@@ -1584,16 +1584,16 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>29.5</v>
+        <v>17.5</v>
       </c>
       <c r="E40" t="n">
-        <v>0.04646765495748104</v>
+        <v>0.00902006196943346</v>
       </c>
       <c r="F40" t="n">
-        <v>-2.066188350836505</v>
+        <v>2.811843450565678</v>
       </c>
       <c r="G40" t="n">
-        <v>0.05653088132823384</v>
+        <v>0.01314181232696556</v>
       </c>
     </row>
     <row r="41">
@@ -1642,16 +1642,16 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0</v>
+        <v>20.5</v>
       </c>
       <c r="E42" t="n">
-        <v>3.0517578125e-05</v>
+        <v>0.01404280667398784</v>
       </c>
       <c r="F42" t="n">
-        <v>-9.470496130340521</v>
+        <v>3.039040638315052</v>
       </c>
       <c r="G42" t="n">
-        <v>1.017288601181338e-07</v>
+        <v>0.008286615044678168</v>
       </c>
     </row>
     <row r="43">
@@ -1671,16 +1671,16 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>6.103515625e-05</v>
       </c>
       <c r="F43" t="n">
-        <v>0</v>
+        <v>7.69545015773808</v>
       </c>
       <c r="G43" t="n">
-        <v>1</v>
+        <v>1.384189718648406e-06</v>
       </c>
     </row>
     <row r="44">
@@ -1758,16 +1758,16 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="E46" t="n">
-        <v>0.00628662109375</v>
+        <v>0.17535400390625</v>
       </c>
       <c r="F46" t="n">
-        <v>-3.075663229507477</v>
+        <v>1.668608286559367</v>
       </c>
       <c r="G46" t="n">
-        <v>0.007690047379809485</v>
+        <v>0.1159283406436272</v>
       </c>
     </row>
     <row r="47">
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E48" t="n">
-        <v>0.009185791015625</v>
+        <v>0.00628662109375</v>
       </c>
       <c r="F48" t="n">
-        <v>-1.723616456583138</v>
+        <v>3.432213477599011</v>
       </c>
       <c r="G48" t="n">
-        <v>0.1053201907118546</v>
+        <v>0.003704622490571183</v>
       </c>
     </row>
     <row r="49">
@@ -1845,16 +1845,16 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E49" t="n">
-        <v>1</v>
+        <v>0.00030517578125</v>
       </c>
       <c r="F49" t="n">
-        <v>0</v>
+        <v>4.354869795379987</v>
       </c>
       <c r="G49" t="n">
-        <v>1</v>
+        <v>0.0005658542849788176</v>
       </c>
     </row>
     <row r="50">
@@ -2918,16 +2918,16 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>66</v>
+        <v>6</v>
       </c>
       <c r="E86" t="n">
-        <v>0.9175629288442165</v>
+        <v>0.001338697889830873</v>
       </c>
       <c r="F86" t="n">
-        <v>0.7254938879651808</v>
+        <v>3.677702566003692</v>
       </c>
       <c r="G86" t="n">
-        <v>0.4793158888196577</v>
+        <v>0.002239059966241018</v>
       </c>
     </row>
     <row r="87">
@@ -2947,16 +2947,16 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>61.5</v>
+        <v>20.5</v>
       </c>
       <c r="E87" t="n">
-        <v>0.7367901810877747</v>
+        <v>0.01397871086028363</v>
       </c>
       <c r="F87" t="n">
-        <v>0.5383001086105844</v>
+        <v>-2.784271303622158</v>
       </c>
       <c r="G87" t="n">
-        <v>0.5982676234947266</v>
+        <v>0.01389351058264812</v>
       </c>
     </row>
     <row r="88">
@@ -2976,16 +2976,16 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>61</v>
+        <v>0.5</v>
       </c>
       <c r="E88" t="n">
-        <v>0.717199905483448</v>
+        <v>0.0004813507574741004</v>
       </c>
       <c r="F88" t="n">
-        <v>0.09215591934378574</v>
+        <v>8.198977631202018</v>
       </c>
       <c r="G88" t="n">
-        <v>0.9277936832871893</v>
+        <v>6.354473091419399e-07</v>
       </c>
     </row>
     <row r="89">
@@ -3005,16 +3005,16 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="E89" t="n">
-        <v>0.8767013015603727</v>
+        <v>3.0517578125e-05</v>
       </c>
       <c r="F89" t="n">
-        <v>0.7885825689571988</v>
+        <v>5.809697973710994</v>
       </c>
       <c r="G89" t="n">
-        <v>0.4426416105898565</v>
+        <v>3.439103369621853e-05</v>
       </c>
     </row>
     <row r="90">
@@ -3846,16 +3846,16 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E118" t="n">
-        <v>3.0517578125e-05</v>
+        <v>6.103515625e-05</v>
       </c>
       <c r="F118" t="n">
-        <v>8.766820066313747</v>
+        <v>6.37548140972848</v>
       </c>
       <c r="G118" t="n">
-        <v>2.740611576655298e-07</v>
+        <v>1.246634039145319e-05</v>
       </c>
     </row>
     <row r="119">
@@ -3875,16 +3875,16 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E119" t="n">
-        <v>0.000213623046875</v>
+        <v>6.103515625e-05</v>
       </c>
       <c r="F119" t="n">
-        <v>3.772039140193199</v>
+        <v>5.479405362348543</v>
       </c>
       <c r="G119" t="n">
-        <v>0.001845813992803375</v>
+        <v>6.345798234782795e-05</v>
       </c>
     </row>
     <row r="120">
@@ -3904,16 +3904,16 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>0</v>
+        <v>44.5</v>
       </c>
       <c r="E120" t="n">
-        <v>3.0517578125e-05</v>
+        <v>0.2243065711972715</v>
       </c>
       <c r="F120" t="n">
-        <v>12.55786324440561</v>
+        <v>1.060450735487672</v>
       </c>
       <c r="G120" t="n">
-        <v>2.31731049642291e-09</v>
+        <v>0.3057170087228476</v>
       </c>
     </row>
     <row r="121">
@@ -3933,16 +3933,16 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="E121" t="n">
-        <v>3.0517578125e-05</v>
+        <v>0.00213623046875</v>
       </c>
       <c r="F121" t="n">
-        <v>8.255384020444454</v>
+        <v>3.740204457992197</v>
       </c>
       <c r="G121" t="n">
-        <v>5.835145404940795e-07</v>
+        <v>0.00197005439477589</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update inter model compare files
</commit_message>
<xml_diff>
--- a/inter_model_compare/Inter_model_Stat_results.xlsx
+++ b/inter_model_compare/Inter_model_Stat_results.xlsx
@@ -485,13 +485,13 @@
         <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0007654126488518396</v>
+        <v>0.0007669773627198459</v>
       </c>
       <c r="F2" t="n">
-        <v>-4.086928883368941</v>
+        <v>-4.078414776588619</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0009716748884118768</v>
+        <v>0.0009886024298329638</v>
       </c>
     </row>
     <row r="3">
@@ -511,16 +511,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>48</v>
+        <v>48.5</v>
       </c>
       <c r="E3" t="n">
-        <v>0.3004880879398838</v>
+        <v>0.3129767043632334</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.9763887227517427</v>
+        <v>-0.9585907606755874</v>
       </c>
       <c r="G3" t="n">
-        <v>0.3443567449283444</v>
+        <v>0.3529620313071024</v>
       </c>
     </row>
     <row r="4">
@@ -540,16 +540,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>24.5</v>
+        <v>25</v>
       </c>
       <c r="E4" t="n">
-        <v>0.021392822265625</v>
+        <v>0.02496337890625</v>
       </c>
       <c r="F4" t="n">
-        <v>-2.957172569384298</v>
+        <v>-2.94826596781852</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0097896561366208</v>
+        <v>0.009968489871660418</v>
       </c>
     </row>
     <row r="5">
@@ -572,13 +572,13 @@
         <v>5</v>
       </c>
       <c r="E5" t="n">
-        <v>0.001116926714212636</v>
+        <v>0.001114781427556677</v>
       </c>
       <c r="F5" t="n">
-        <v>3.571183494257071</v>
+        <v>3.576439583178546</v>
       </c>
       <c r="G5" t="n">
-        <v>0.002785518587903024</v>
+        <v>0.002755649040233676</v>
       </c>
     </row>
     <row r="6">
@@ -633,10 +633,10 @@
         <v>0.01396270726023798</v>
       </c>
       <c r="F7" t="n">
-        <v>-2.547544506144599</v>
+        <v>-2.550320957269724</v>
       </c>
       <c r="G7" t="n">
-        <v>0.02230628118138613</v>
+        <v>0.02218384902950845</v>
       </c>
     </row>
     <row r="8">
@@ -833,13 +833,13 @@
         <v>19.5</v>
       </c>
       <c r="E14" t="n">
-        <v>0.01211715774633701</v>
+        <v>0.01213155109444909</v>
       </c>
       <c r="F14" t="n">
-        <v>-2.935709877698803</v>
+        <v>-2.937075494962023</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0102260483109191</v>
+        <v>0.01019772305106727</v>
       </c>
     </row>
     <row r="15">
@@ -865,10 +865,10 @@
         <v>0.1473894450908428</v>
       </c>
       <c r="F15" t="n">
-        <v>-1.215785317142074</v>
+        <v>-1.220346319907168</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2428550481303261</v>
+        <v>0.241172128119603</v>
       </c>
     </row>
     <row r="16">
@@ -894,10 +894,10 @@
         <v>0.1033498116616814</v>
       </c>
       <c r="F16" t="n">
-        <v>-1.695482055506622</v>
+        <v>-1.700672238529259</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1106351453286317</v>
+        <v>0.1096374287655518</v>
       </c>
     </row>
     <row r="17">
@@ -923,10 +923,10 @@
         <v>0.2662505867944568</v>
       </c>
       <c r="F17" t="n">
-        <v>1.510831688064607</v>
+        <v>1.512890179799334</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1516089640136974</v>
+        <v>0.1510895831307116</v>
       </c>
     </row>
     <row r="18">
@@ -981,10 +981,10 @@
         <v>0.5871071989491958</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.9690867357995401</v>
+        <v>-0.9716794572702423</v>
       </c>
       <c r="G19" t="n">
-        <v>0.3478692472343407</v>
+        <v>0.3466191943490792</v>
       </c>
     </row>
     <row r="20">
@@ -1010,10 +1010,10 @@
         <v>0.0026988080978068</v>
       </c>
       <c r="F20" t="n">
-        <v>-3.493727181804557</v>
+        <v>-3.498138901261981</v>
       </c>
       <c r="G20" t="n">
-        <v>0.003265291852510518</v>
+        <v>0.003235864983673819</v>
       </c>
     </row>
     <row r="21">
@@ -1033,16 +1033,16 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>65.5</v>
+        <v>66</v>
       </c>
       <c r="E21" t="n">
-        <v>0.899932861328125</v>
+        <v>0.93988037109375</v>
       </c>
       <c r="F21" t="n">
-        <v>0.6455920276469586</v>
+        <v>0.6484561034536114</v>
       </c>
       <c r="G21" t="n">
-        <v>0.5282965206410231</v>
+        <v>0.5264932825354662</v>
       </c>
     </row>
     <row r="22">
@@ -1097,10 +1097,10 @@
         <v>0.00042724609375</v>
       </c>
       <c r="F23" t="n">
-        <v>3.172362574427624</v>
+        <v>3.181751922145879</v>
       </c>
       <c r="G23" t="n">
-        <v>0.006310940059913092</v>
+        <v>0.006190834700855789</v>
       </c>
     </row>
     <row r="24">
@@ -1126,10 +1126,10 @@
         <v>0.013092041015625</v>
       </c>
       <c r="F24" t="n">
-        <v>2.486130099681526</v>
+        <v>2.496059562647546</v>
       </c>
       <c r="G24" t="n">
-        <v>0.02518550181416795</v>
+        <v>0.02469710610928627</v>
       </c>
     </row>
     <row r="25">
@@ -1155,10 +1155,10 @@
         <v>0.00762939453125</v>
       </c>
       <c r="F25" t="n">
-        <v>-2.561075546215715</v>
+        <v>-2.566977652551726</v>
       </c>
       <c r="G25" t="n">
-        <v>0.0217156520653525</v>
+        <v>0.02146274350432676</v>
       </c>
     </row>
     <row r="26">
@@ -1181,13 +1181,13 @@
         <v>6.5</v>
       </c>
       <c r="E26" t="n">
-        <v>0.001456153717910081</v>
+        <v>0.001464210818129427</v>
       </c>
       <c r="F26" t="n">
-        <v>-2.756907783072998</v>
+        <v>-2.793546191675929</v>
       </c>
       <c r="G26" t="n">
-        <v>0.01468073907505756</v>
+        <v>0.01363610083426323</v>
       </c>
     </row>
     <row r="27">
@@ -1213,10 +1213,10 @@
         <v>0.007724233637416746</v>
       </c>
       <c r="F27" t="n">
-        <v>-3.010098070412778</v>
+        <v>-3.011204149188707</v>
       </c>
       <c r="G27" t="n">
-        <v>0.008790093097708975</v>
+        <v>0.008770310746133212</v>
       </c>
     </row>
     <row r="28">
@@ -1236,16 +1236,16 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>52.5</v>
+        <v>51.5</v>
       </c>
       <c r="E28" t="n">
-        <v>0.433197021484375</v>
+        <v>0.40374755859375</v>
       </c>
       <c r="F28" t="n">
-        <v>-1.470387340513864</v>
+        <v>-1.476692568385537</v>
       </c>
       <c r="G28" t="n">
-        <v>0.1621208233067553</v>
+        <v>0.1604431421947784</v>
       </c>
     </row>
     <row r="29">
@@ -1271,10 +1271,10 @@
         <v>0.021392822265625</v>
       </c>
       <c r="F29" t="n">
-        <v>-1.664837300219328</v>
+        <v>-1.615977004795708</v>
       </c>
       <c r="G29" t="n">
-        <v>0.1166883803046404</v>
+        <v>0.1269320316665925</v>
       </c>
     </row>
     <row r="30">
@@ -1294,16 +1294,16 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>27</v>
+        <v>26.5</v>
       </c>
       <c r="E30" t="n">
         <v>0.033538818359375</v>
       </c>
       <c r="F30" t="n">
-        <v>2.129538870678781</v>
+        <v>2.137271066714171</v>
       </c>
       <c r="G30" t="n">
-        <v>0.05018088582646035</v>
+        <v>0.04945257453954477</v>
       </c>
     </row>
     <row r="31">
@@ -1329,10 +1329,10 @@
         <v>0.010986328125</v>
       </c>
       <c r="F31" t="n">
-        <v>2.97869377386183</v>
+        <v>2.977974048298377</v>
       </c>
       <c r="G31" t="n">
-        <v>0.009370417962060751</v>
+        <v>0.00938414939969273</v>
       </c>
     </row>
     <row r="32">
@@ -1358,10 +1358,10 @@
         <v>0.0008523328835916312</v>
       </c>
       <c r="F32" t="n">
-        <v>-4.121464683874558</v>
+        <v>-4.123858893324051</v>
       </c>
       <c r="G32" t="n">
-        <v>0.000905980059884941</v>
+        <v>0.0009015967985754488</v>
       </c>
     </row>
     <row r="33">
@@ -1445,10 +1445,10 @@
         <v>0.002478331942743607</v>
       </c>
       <c r="F35" t="n">
-        <v>2.7908305332692</v>
+        <v>2.793080578732155</v>
       </c>
       <c r="G35" t="n">
-        <v>0.01371098595327495</v>
+        <v>0.01364891196266068</v>
       </c>
     </row>
     <row r="36">
@@ -1474,10 +1474,10 @@
         <v>0.815942129589875</v>
       </c>
       <c r="F36" t="n">
-        <v>-0.286192865876731</v>
+        <v>-0.2830289629422025</v>
       </c>
       <c r="G36" t="n">
-        <v>0.7786451558117076</v>
+        <v>0.7810231911668137</v>
       </c>
     </row>
     <row r="37">
@@ -1532,10 +1532,10 @@
         <v>0.1705987715966291</v>
       </c>
       <c r="F38" t="n">
-        <v>1.697751230832075</v>
+        <v>1.673235300338404</v>
       </c>
       <c r="G38" t="n">
-        <v>0.1101979704029439</v>
+        <v>0.1150016293170417</v>
       </c>
     </row>
     <row r="39">
@@ -1561,10 +1561,10 @@
         <v>0.04646765495748104</v>
       </c>
       <c r="F39" t="n">
-        <v>-2.066188350836505</v>
+        <v>-2.073630224294672</v>
       </c>
       <c r="G39" t="n">
-        <v>0.05653088132823384</v>
+        <v>0.05574844225696523</v>
       </c>
     </row>
     <row r="40">
@@ -1590,10 +1590,10 @@
         <v>0.00902006196943346</v>
       </c>
       <c r="F40" t="n">
-        <v>2.811843450565678</v>
+        <v>2.815102243875117</v>
       </c>
       <c r="G40" t="n">
-        <v>0.01314181232696556</v>
+        <v>0.01305562559524748</v>
       </c>
     </row>
     <row r="41">
@@ -1619,10 +1619,10 @@
         <v>3.0517578125e-05</v>
       </c>
       <c r="F41" t="n">
-        <v>-9.470496130340521</v>
+        <v>-9.395243274694424</v>
       </c>
       <c r="G41" t="n">
-        <v>1.017288601181338e-07</v>
+        <v>1.128109378972695e-07</v>
       </c>
     </row>
     <row r="42">
@@ -1648,10 +1648,10 @@
         <v>0.01404280667398784</v>
       </c>
       <c r="F42" t="n">
-        <v>3.039040638315052</v>
+        <v>3.063270067026647</v>
       </c>
       <c r="G42" t="n">
-        <v>0.008286615044678168</v>
+        <v>0.007887032605941381</v>
       </c>
     </row>
     <row r="43">
@@ -1677,10 +1677,10 @@
         <v>6.103515625e-05</v>
       </c>
       <c r="F43" t="n">
-        <v>7.69545015773808</v>
+        <v>7.723964739458935</v>
       </c>
       <c r="G43" t="n">
-        <v>1.384189718648406e-06</v>
+        <v>1.323360142336815e-06</v>
       </c>
     </row>
     <row r="44">
@@ -1706,10 +1706,10 @@
         <v>0.007744704507695919</v>
       </c>
       <c r="F44" t="n">
-        <v>-2.738088330092935</v>
+        <v>-2.794144867557283</v>
       </c>
       <c r="G44" t="n">
-        <v>0.01524709309481322</v>
+        <v>0.01361964571148231</v>
       </c>
     </row>
     <row r="45">
@@ -1735,10 +1735,10 @@
         <v>0.00628662109375</v>
       </c>
       <c r="F45" t="n">
-        <v>-3.075663229507477</v>
+        <v>-3.07624202789817</v>
       </c>
       <c r="G45" t="n">
-        <v>0.007690047379809485</v>
+        <v>0.007680967040506912</v>
       </c>
     </row>
     <row r="46">
@@ -1764,10 +1764,10 @@
         <v>0.17535400390625</v>
       </c>
       <c r="F46" t="n">
-        <v>1.668608286559367</v>
+        <v>1.665083641370279</v>
       </c>
       <c r="G46" t="n">
-        <v>0.1159283406436272</v>
+        <v>0.1166385990882629</v>
       </c>
     </row>
     <row r="47">
@@ -1793,10 +1793,10 @@
         <v>0.009185791015625</v>
       </c>
       <c r="F47" t="n">
-        <v>-1.723616456583138</v>
+        <v>-1.697831493409904</v>
       </c>
       <c r="G47" t="n">
-        <v>0.1053201907118546</v>
+        <v>0.1101825347383526</v>
       </c>
     </row>
     <row r="48">
@@ -1822,10 +1822,10 @@
         <v>0.00628662109375</v>
       </c>
       <c r="F48" t="n">
-        <v>3.432213477599011</v>
+        <v>3.446849069267472</v>
       </c>
       <c r="G48" t="n">
-        <v>0.003704622490571183</v>
+        <v>0.003595012648220033</v>
       </c>
     </row>
     <row r="49">
@@ -1851,10 +1851,10 @@
         <v>0.00030517578125</v>
       </c>
       <c r="F49" t="n">
-        <v>4.354869795379987</v>
+        <v>4.352355110205695</v>
       </c>
       <c r="G49" t="n">
-        <v>0.0005658542849788176</v>
+        <v>0.0005687171427868268</v>
       </c>
     </row>
     <row r="50">
@@ -1874,16 +1874,16 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>64.5</v>
+        <v>64</v>
       </c>
       <c r="E50" t="n">
-        <v>0.856287680138486</v>
+        <v>0.8360576167309932</v>
       </c>
       <c r="F50" t="n">
-        <v>-0.4491415610471458</v>
+        <v>-0.4482998003163862</v>
       </c>
       <c r="G50" t="n">
-        <v>0.6597507316026566</v>
+        <v>0.6603444336584146</v>
       </c>
     </row>
     <row r="51">
@@ -1903,16 +1903,16 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>66</v>
+        <v>65.5</v>
       </c>
       <c r="E51" t="n">
-        <v>0.9176178742687193</v>
+        <v>0.8971082840978747</v>
       </c>
       <c r="F51" t="n">
-        <v>-0.1113931750883391</v>
+        <v>-0.1146112697834352</v>
       </c>
       <c r="G51" t="n">
-        <v>0.9127814647258554</v>
+        <v>0.9102733389299482</v>
       </c>
     </row>
     <row r="52">
@@ -1932,16 +1932,16 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>19</v>
+        <v>19.5</v>
       </c>
       <c r="E52" t="n">
-        <v>0.01124470406185358</v>
+        <v>0.01211715774633701</v>
       </c>
       <c r="F52" t="n">
-        <v>3.22510880374006</v>
+        <v>3.223219130503807</v>
       </c>
       <c r="G52" t="n">
-        <v>0.005664945732526467</v>
+        <v>0.005686914543073384</v>
       </c>
     </row>
     <row r="53">
@@ -1967,10 +1967,10 @@
         <v>0.7959205023955187</v>
       </c>
       <c r="F53" t="n">
-        <v>0.1848768099869045</v>
+        <v>0.1820567213777432</v>
       </c>
       <c r="G53" t="n">
-        <v>0.8558021231811626</v>
+        <v>0.8579757352081941</v>
       </c>
     </row>
     <row r="54">
@@ -1996,10 +1996,10 @@
         <v>9.1552734375e-05</v>
       </c>
       <c r="F54" t="n">
-        <v>4.455523276165934</v>
+        <v>4.452411030527481</v>
       </c>
       <c r="G54" t="n">
-        <v>0.0004625788222528388</v>
+        <v>0.0004654635426867107</v>
       </c>
     </row>
     <row r="55">
@@ -2228,10 +2228,10 @@
         <v>0.00294660290680535</v>
       </c>
       <c r="F62" t="n">
-        <v>4.322153830051519</v>
+        <v>4.302751009536563</v>
       </c>
       <c r="G62" t="n">
-        <v>0.0006042793807634956</v>
+        <v>0.0006283175700818884</v>
       </c>
     </row>
     <row r="63">
@@ -2257,10 +2257,10 @@
         <v>6.103515625e-05</v>
       </c>
       <c r="F63" t="n">
-        <v>-5.870659912881088</v>
+        <v>-5.849700936616495</v>
       </c>
       <c r="G63" t="n">
-        <v>3.07639970710808e-05</v>
+        <v>3.196383644598586e-05</v>
       </c>
     </row>
     <row r="64">
@@ -2286,10 +2286,10 @@
         <v>0.006633375463483006</v>
       </c>
       <c r="F64" t="n">
-        <v>3.617522137535851</v>
+        <v>3.605569555391973</v>
       </c>
       <c r="G64" t="n">
-        <v>0.002532996978543799</v>
+        <v>0.002595843526420557</v>
       </c>
     </row>
     <row r="65">
@@ -2315,10 +2315,10 @@
         <v>3.0517578125e-05</v>
       </c>
       <c r="F65" t="n">
-        <v>-13.20993937012326</v>
+        <v>-13.298770106964</v>
       </c>
       <c r="G65" t="n">
-        <v>1.150716630898938e-09</v>
+        <v>1.048438221532935e-09</v>
       </c>
     </row>
     <row r="66">
@@ -2373,10 +2373,10 @@
         <v>3.0517578125e-05</v>
       </c>
       <c r="F67" t="n">
-        <v>13.50982914556335</v>
+        <v>13.53227825714303</v>
       </c>
       <c r="G67" t="n">
-        <v>8.421904161561828e-10</v>
+        <v>8.2293708964579e-10</v>
       </c>
     </row>
     <row r="68">
@@ -2431,10 +2431,10 @@
         <v>0.1873117012677681</v>
       </c>
       <c r="F69" t="n">
-        <v>-1.228989938675668</v>
+        <v>-1.226459201347515</v>
       </c>
       <c r="G69" t="n">
-        <v>0.2380076529570154</v>
+        <v>0.2389308075024994</v>
       </c>
     </row>
     <row r="70">
@@ -2454,16 +2454,16 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="E70" t="n">
-        <v>0.001121225500855849</v>
+        <v>0.001025241598635927</v>
       </c>
       <c r="F70" t="n">
-        <v>3.572075069145006</v>
+        <v>3.581537458124911</v>
       </c>
       <c r="G70" t="n">
-        <v>0.00278042911244368</v>
+        <v>0.002726985782020555</v>
       </c>
     </row>
     <row r="71">
@@ -2489,10 +2489,10 @@
         <v>0.00762939453125</v>
       </c>
       <c r="F71" t="n">
-        <v>-2.270756787710648</v>
+        <v>-2.268442183679862</v>
       </c>
       <c r="G71" t="n">
-        <v>0.03832686588161546</v>
+        <v>0.03849807515186269</v>
       </c>
     </row>
     <row r="72">
@@ -2518,10 +2518,10 @@
         <v>0.00335693359375</v>
       </c>
       <c r="F72" t="n">
-        <v>2.890461404700636</v>
+        <v>2.898596468311895</v>
       </c>
       <c r="G72" t="n">
-        <v>0.01120937437769266</v>
+        <v>0.01102601650573136</v>
       </c>
     </row>
     <row r="73">
@@ -2547,10 +2547,10 @@
         <v>0.000213623046875</v>
       </c>
       <c r="F73" t="n">
-        <v>4.856356356109245</v>
+        <v>4.858735245387731</v>
       </c>
       <c r="G73" t="n">
-        <v>0.0002094525864991406</v>
+        <v>0.000208480967733761</v>
       </c>
     </row>
     <row r="74">
@@ -2576,10 +2576,10 @@
         <v>0.02613360703702765</v>
       </c>
       <c r="F74" t="n">
-        <v>1.97985420168623</v>
+        <v>1.987557350732113</v>
       </c>
       <c r="G74" t="n">
-        <v>0.06637143292373512</v>
+        <v>0.06543393723369045</v>
       </c>
     </row>
     <row r="75">
@@ -2634,10 +2634,10 @@
         <v>0.8563589864870352</v>
       </c>
       <c r="F76" t="n">
-        <v>0.2332754649718186</v>
+        <v>0.2312535779583915</v>
       </c>
       <c r="G76" t="n">
-        <v>0.8187009605105208</v>
+        <v>0.8202426290787704</v>
       </c>
     </row>
     <row r="77">
@@ -2692,10 +2692,10 @@
         <v>3.0517578125e-05</v>
       </c>
       <c r="F78" t="n">
-        <v>5.512586233822182</v>
+        <v>5.448867926179909</v>
       </c>
       <c r="G78" t="n">
-        <v>5.963117636566023e-05</v>
+        <v>6.720521289353249e-05</v>
       </c>
     </row>
     <row r="79">
@@ -2721,10 +2721,10 @@
         <v>0.7760323448046139</v>
       </c>
       <c r="F79" t="n">
-        <v>0.3790373225584922</v>
+        <v>0.3759705168569499</v>
       </c>
       <c r="G79" t="n">
-        <v>0.7099717461517161</v>
+        <v>0.7122029567640535</v>
       </c>
     </row>
     <row r="80">
@@ -2750,10 +2750,10 @@
         <v>3.0517578125e-05</v>
       </c>
       <c r="F80" t="n">
-        <v>7.221469448742603</v>
+        <v>7.200281255252341</v>
       </c>
       <c r="G80" t="n">
-        <v>2.967033112860932e-06</v>
+        <v>3.072018249146425e-06</v>
       </c>
     </row>
     <row r="81">
@@ -2779,10 +2779,10 @@
         <v>3.0517578125e-05</v>
       </c>
       <c r="F81" t="n">
-        <v>5.566820324197988</v>
+        <v>5.529840569034401</v>
       </c>
       <c r="G81" t="n">
-        <v>5.388372436007893e-05</v>
+        <v>5.773664111133436e-05</v>
       </c>
     </row>
     <row r="82">
@@ -2802,16 +2802,16 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>13.5</v>
+        <v>13</v>
       </c>
       <c r="E82" t="n">
-        <v>0.00475989564421327</v>
+        <v>0.004408971264023412</v>
       </c>
       <c r="F82" t="n">
-        <v>-3.396668753441344</v>
+        <v>-3.407555087060483</v>
       </c>
       <c r="G82" t="n">
-        <v>0.003984928857416943</v>
+        <v>0.003896900121966295</v>
       </c>
     </row>
     <row r="83">
@@ -2866,10 +2866,10 @@
         <v>0.6048534511043099</v>
       </c>
       <c r="F84" t="n">
-        <v>-0.9266629451993296</v>
+        <v>-0.9251357122588485</v>
       </c>
       <c r="G84" t="n">
-        <v>0.3687720885607469</v>
+        <v>0.369540353214851</v>
       </c>
     </row>
     <row r="85">
@@ -2895,10 +2895,10 @@
         <v>0.001312255859375</v>
       </c>
       <c r="F85" t="n">
-        <v>-2.849587477872165</v>
+        <v>-2.859018879746591</v>
       </c>
       <c r="G85" t="n">
-        <v>0.01217664744715107</v>
+        <v>0.01194647426615434</v>
       </c>
     </row>
     <row r="86">
@@ -2921,13 +2921,13 @@
         <v>6</v>
       </c>
       <c r="E86" t="n">
-        <v>0.001338697889830873</v>
+        <v>0.001341196663435169</v>
       </c>
       <c r="F86" t="n">
-        <v>3.677702566003692</v>
+        <v>3.66683433553598</v>
       </c>
       <c r="G86" t="n">
-        <v>0.002239059966241018</v>
+        <v>0.002289480511912319</v>
       </c>
     </row>
     <row r="87">
@@ -2982,10 +2982,10 @@
         <v>0.0004813507574741004</v>
       </c>
       <c r="F88" t="n">
-        <v>8.198977631202018</v>
+        <v>8.224368258558318</v>
       </c>
       <c r="G88" t="n">
-        <v>6.354473091419399e-07</v>
+        <v>6.114924812587537e-07</v>
       </c>
     </row>
     <row r="89">
@@ -3011,10 +3011,10 @@
         <v>3.0517578125e-05</v>
       </c>
       <c r="F89" t="n">
-        <v>5.809697973710994</v>
+        <v>5.802375492072645</v>
       </c>
       <c r="G89" t="n">
-        <v>3.439103369621853e-05</v>
+        <v>3.48557090851392e-05</v>
       </c>
     </row>
     <row r="90">
@@ -3040,10 +3040,10 @@
         <v>0.001007080078125</v>
       </c>
       <c r="F90" t="n">
-        <v>4.569837548965428</v>
+        <v>4.568182478827398</v>
       </c>
       <c r="G90" t="n">
-        <v>0.0003683854859449038</v>
+        <v>0.0003695984166753593</v>
       </c>
     </row>
     <row r="91">
@@ -3098,10 +3098,10 @@
         <v>0.001472296771329153</v>
       </c>
       <c r="F92" t="n">
-        <v>4.260802851177417</v>
+        <v>4.252967508032811</v>
       </c>
       <c r="G92" t="n">
-        <v>0.0006836815065689365</v>
+        <v>0.0006945624105245075</v>
       </c>
     </row>
     <row r="93">
@@ -3127,10 +3127,10 @@
         <v>0.001312255859375</v>
       </c>
       <c r="F93" t="n">
-        <v>3.771001804298804</v>
+        <v>3.767552315851426</v>
       </c>
       <c r="G93" t="n">
-        <v>0.00184973498383166</v>
+        <v>0.001862834153073368</v>
       </c>
     </row>
     <row r="94">
@@ -3156,10 +3156,10 @@
         <v>3.0517578125e-05</v>
       </c>
       <c r="F94" t="n">
-        <v>8.546881076105329</v>
+        <v>8.542992042055397</v>
       </c>
       <c r="G94" t="n">
-        <v>3.77874597141247e-07</v>
+        <v>3.800462428836253e-07</v>
       </c>
     </row>
     <row r="95">
@@ -3214,10 +3214,10 @@
         <v>3.0517578125e-05</v>
       </c>
       <c r="F96" t="n">
-        <v>15.65507996779514</v>
+        <v>15.69701341518648</v>
       </c>
       <c r="G96" t="n">
-        <v>1.060163069705735e-10</v>
+        <v>1.020682040588237e-10</v>
       </c>
     </row>
     <row r="97">
@@ -3243,10 +3243,10 @@
         <v>3.0517578125e-05</v>
       </c>
       <c r="F97" t="n">
-        <v>10.11951793356532</v>
+        <v>10.12372974123173</v>
       </c>
       <c r="G97" t="n">
-        <v>4.272827530406719e-08</v>
+        <v>4.249430377363232e-08</v>
       </c>
     </row>
     <row r="98">
@@ -3266,16 +3266,16 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>8.5</v>
+        <v>9</v>
       </c>
       <c r="E98" t="n">
         <v>0.001007080078125</v>
       </c>
       <c r="F98" t="n">
-        <v>4.563044692890468</v>
+        <v>4.539361844879424</v>
       </c>
       <c r="G98" t="n">
-        <v>0.0003733898489325161</v>
+        <v>0.0003913893104088936</v>
       </c>
     </row>
     <row r="99">
@@ -3330,10 +3330,10 @@
         <v>0.1330799252012172</v>
       </c>
       <c r="F100" t="n">
-        <v>-1.828825788693395</v>
+        <v>-1.819984439955779</v>
       </c>
       <c r="G100" t="n">
-        <v>0.08737681238794072</v>
+        <v>0.08877302601894407</v>
       </c>
     </row>
     <row r="101">
@@ -3359,10 +3359,10 @@
         <v>0.00628662109375</v>
       </c>
       <c r="F101" t="n">
-        <v>3.446404165099607</v>
+        <v>3.442477440104279</v>
       </c>
       <c r="G101" t="n">
-        <v>0.003598296386048426</v>
+        <v>0.003627408995563914</v>
       </c>
     </row>
     <row r="102">
@@ -3388,10 +3388,10 @@
         <v>3.0517578125e-05</v>
       </c>
       <c r="F102" t="n">
-        <v>8.213799058051645</v>
+        <v>8.213396402035487</v>
       </c>
       <c r="G102" t="n">
-        <v>6.213463712832105e-07</v>
+        <v>6.217250670725113e-07</v>
       </c>
     </row>
     <row r="103">
@@ -3446,10 +3446,10 @@
         <v>0.0004824029369617037</v>
       </c>
       <c r="F104" t="n">
-        <v>8.851537430636238</v>
+        <v>8.823652499611759</v>
       </c>
       <c r="G104" t="n">
-        <v>2.425273351175623e-07</v>
+        <v>2.524614306000734e-07</v>
       </c>
     </row>
     <row r="105">
@@ -3475,10 +3475,10 @@
         <v>3.0517578125e-05</v>
       </c>
       <c r="F105" t="n">
-        <v>7.639694625603002</v>
+        <v>7.646354153483629</v>
       </c>
       <c r="G105" t="n">
-        <v>1.51178345755484e-06</v>
+        <v>1.495913868519253e-06</v>
       </c>
     </row>
     <row r="106">
@@ -3556,16 +3556,16 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E108" t="n">
-        <v>0.02984575932785975</v>
+        <v>0.02615862349838189</v>
       </c>
       <c r="F108" t="n">
-        <v>2.703085344169733</v>
+        <v>2.700365911381575</v>
       </c>
       <c r="G108" t="n">
-        <v>0.01635726306614604</v>
+        <v>0.016446713582909</v>
       </c>
     </row>
     <row r="109">
@@ -3585,16 +3585,16 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>22.5</v>
+        <v>23.5</v>
       </c>
       <c r="E109" t="n">
-        <v>0.01863520888400527</v>
+        <v>0.02138935776678794</v>
       </c>
       <c r="F109" t="n">
-        <v>2.811777120608145</v>
+        <v>2.808856117227373</v>
       </c>
       <c r="G109" t="n">
-        <v>0.0131435723196686</v>
+        <v>0.01322130573030058</v>
       </c>
     </row>
     <row r="110">
@@ -3620,10 +3620,10 @@
         <v>3.0517578125e-05</v>
       </c>
       <c r="F110" t="n">
-        <v>6.197242073408737</v>
+        <v>6.181917906910431</v>
       </c>
       <c r="G110" t="n">
-        <v>1.708090425857789e-05</v>
+        <v>1.755329476925826e-05</v>
       </c>
     </row>
     <row r="111">
@@ -3649,10 +3649,10 @@
         <v>0.003199482998392444</v>
       </c>
       <c r="F111" t="n">
-        <v>2.728165309707786</v>
+        <v>2.730746465603809</v>
       </c>
       <c r="G111" t="n">
-        <v>0.01555418304485223</v>
+        <v>0.0154737319338741</v>
       </c>
     </row>
     <row r="112">
@@ -3678,10 +3678,10 @@
         <v>6.103515625e-05</v>
       </c>
       <c r="F112" t="n">
-        <v>7.07704637332493</v>
+        <v>7.111227580176263</v>
       </c>
       <c r="G112" t="n">
-        <v>3.765058376917888e-06</v>
+        <v>3.557776535916903e-06</v>
       </c>
     </row>
     <row r="113">
@@ -3707,10 +3707,10 @@
         <v>3.0517578125e-05</v>
       </c>
       <c r="F113" t="n">
-        <v>7.773375314868292</v>
+        <v>7.808487782220144</v>
       </c>
       <c r="G113" t="n">
-        <v>1.224515440912796e-06</v>
+        <v>1.159012850340474e-06</v>
       </c>
     </row>
     <row r="114">
@@ -3736,10 +3736,10 @@
         <v>0.000152587890625</v>
       </c>
       <c r="F114" t="n">
-        <v>6.415729574100197</v>
+        <v>6.394471636787744</v>
       </c>
       <c r="G114" t="n">
-        <v>1.16176355947338e-05</v>
+        <v>1.205810161904097e-05</v>
       </c>
     </row>
     <row r="115">
@@ -3794,10 +3794,10 @@
         <v>0.16239223764448</v>
       </c>
       <c r="F116" t="n">
-        <v>-1.555537203491424</v>
+        <v>-1.549497936192815</v>
       </c>
       <c r="G116" t="n">
-        <v>0.1406613519354034</v>
+        <v>0.1421000517578911</v>
       </c>
     </row>
     <row r="117">
@@ -3823,10 +3823,10 @@
         <v>6.103515625e-05</v>
       </c>
       <c r="F117" t="n">
-        <v>6.787676003124161</v>
+        <v>6.791109305120488</v>
       </c>
       <c r="G117" t="n">
-        <v>6.119411071907829e-06</v>
+        <v>6.083843346245367e-06</v>
       </c>
     </row>
     <row r="118">
@@ -3852,10 +3852,10 @@
         <v>6.103515625e-05</v>
       </c>
       <c r="F118" t="n">
-        <v>6.37548140972848</v>
+        <v>6.37800890218489</v>
       </c>
       <c r="G118" t="n">
-        <v>1.246634039145319e-05</v>
+        <v>1.24111831942265e-05</v>
       </c>
     </row>
     <row r="119">
@@ -3910,10 +3910,10 @@
         <v>0.2243065711972715</v>
       </c>
       <c r="F120" t="n">
-        <v>1.060450735487672</v>
+        <v>1.066545549192049</v>
       </c>
       <c r="G120" t="n">
-        <v>0.3057170087228476</v>
+        <v>0.303043378071447</v>
       </c>
     </row>
     <row r="121">
@@ -3939,10 +3939,10 @@
         <v>0.00213623046875</v>
       </c>
       <c r="F121" t="n">
-        <v>3.740204457992197</v>
+        <v>3.744841104979093</v>
       </c>
       <c r="G121" t="n">
-        <v>0.00197005439477589</v>
+        <v>0.001951447107610953</v>
       </c>
     </row>
   </sheetData>

</xml_diff>